<commit_message>
Phase II Ticketing Reporting Remediation Complete
- Modernized ticketing documentation
- Reclassified severity framework as governance artifact
- Archived historical observations v1
- Updated lifecycle workflow
- Updated subsystem README
- Validated schema and relational model alignment
- Finalized ticket reporting workbook
</commit_message>
<xml_diff>
--- a/ticketing-system/reporting-and-kpis/ticket-analysis-v1.xlsx
+++ b/ticketing-system/reporting-and-kpis/ticket-analysis-v1.xlsx
@@ -741,10 +741,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -810,54 +810,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="0.59999389629810485"/>
@@ -879,76 +831,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="0.59999389629810485"/>
@@ -976,6 +858,57 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <left style="thin">
           <color indexed="64"/>
@@ -1013,6 +946,76 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="0.59999389629810485"/>
@@ -1032,9 +1035,6 @@
           <bgColor theme="9" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -2703,244 +2703,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4283C0DB-D316-4062-937D-7849D5F5D8B6}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="20">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="9"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Ticket Count" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="21">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="20">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="19">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="18">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="17">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="16">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="15">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="14">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="9" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="13">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3826521D-55DC-44D0-9B2F-69FA4EC77E75}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
-  <location ref="A5:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="20">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="7">
-        <item x="3"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Ticket Count" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="30">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="29">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="28">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="27">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="26">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="25">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="24">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="23">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="5" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="22">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D3E0EE18-22CF-48BF-8A21-FC3CFB9322C4}" name="PivotTable14" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I5:L10" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="20">
@@ -3015,42 +2777,42 @@
     <dataField name="Ticket Count" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="10">
-    <format dxfId="40">
+    <format dxfId="22">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="17" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="19">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="18">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="17" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="15">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="13">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -3066,7 +2828,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0612E683-BE2F-4DB1-B66C-F4A6084D6199}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E18:F20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="20">
@@ -3106,6 +2868,212 @@
     </i>
     <i>
       <x v="1"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Ticket Count" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="31">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="30">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="28">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="26">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="25">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C81B2F50-164C-4AF1-98DA-5D67B6FE9F52}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A18:B21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="20">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item n="SLA Not Met" x="1"/>
+        <item n="SLA Met" x="0"/>
+        <item n="Open / Unresolved" x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="17"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Ticket Count" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="40">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="39">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="38">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="37">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="36">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="35">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="34">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="33">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="17" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4283C0DB-D316-4062-937D-7849D5F5D8B6}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="20">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="9"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
     </i>
   </rowItems>
   <colItems count="1">
@@ -3139,7 +3107,7 @@
     <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="11" count="0"/>
+          <reference field="9" count="0"/>
         </references>
       </pivotArea>
     </format>
@@ -3160,41 +3128,56 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C81B2F50-164C-4AF1-98DA-5D67B6FE9F52}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A18:B21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3826521D-55DC-44D0-9B2F-69FA4EC77E75}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" showHeaders="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+  <location ref="A5:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="20">
     <pivotField dataField="1" showAll="0"/>
     <pivotField numFmtId="22" showAll="0"/>
     <pivotField numFmtId="22" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item n="SLA Not Met" x="1"/>
-        <item n="SLA Met" x="0"/>
-        <item n="Open / Unresolved" x="2"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="7">
+        <item x="3"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="5"/>
+        <item x="1"/>
         <item t="default"/>
       </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
     </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
-    <field x="17"/>
+    <field x="5"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="6">
+    <i>
+      <x v="5"/>
+    </i>
     <i>
       <x/>
     </i>
@@ -3203,6 +3186,12 @@
     </i>
     <i>
       <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
     </i>
   </rowItems>
   <colItems count="1">
@@ -3236,7 +3225,7 @@
     <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="17" count="0"/>
+          <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
@@ -3244,6 +3233,17 @@
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -3703,12 +3703,12 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
     </row>
     <row r="36" spans="1:4" s="26" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
@@ -3940,20 +3940,20 @@
       </c>
     </row>
     <row r="13" spans="1:12" ht="74.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="B13" s="28"/>
-      <c r="E13" s="28" t="s">
+      <c r="B13" s="27"/>
+      <c r="E13" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="F13" s="28"/>
-      <c r="I13" s="28" t="s">
+      <c r="F13" s="27"/>
+      <c r="I13" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="J13" s="28"/>
-      <c r="K13" s="28"/>
-      <c r="L13" s="28"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
@@ -4015,14 +4015,14 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="E23" s="28" t="s">
+      <c r="B23" s="27"/>
+      <c r="E23" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="F23" s="28"/>
+      <c r="F23" s="27"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>

</xml_diff>